<commit_message>
time record update +1 hour
</commit_message>
<xml_diff>
--- a/misc/record/Time and Payment.xlsx
+++ b/misc/record/Time and Payment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/Documents/GitHub/Fortune500_SDG_Analysis/misc/record/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABB49D5E-41E5-954D-83EA-3B7212485997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{174B7B65-A31E-0B44-B1FD-0295D3101082}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20" yWindow="980" windowWidth="27040" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-31420" yWindow="2880" windowWidth="27040" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="36">
   <si>
     <t>Date</t>
   </si>
@@ -1533,7 +1533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E117"/>
+  <dimension ref="A1:E125"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="6" width="12.6640625" style="1" customWidth="1"/>
@@ -3211,10 +3211,14 @@
       <c r="E112" s="24"/>
     </row>
     <row r="113" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A113" s="24"/>
+      <c r="A113" s="28">
+        <v>46178</v>
+      </c>
       <c r="B113" s="24"/>
       <c r="C113" s="24"/>
-      <c r="D113" s="24"/>
+      <c r="D113" s="30" t="s">
+        <v>30</v>
+      </c>
       <c r="E113" s="24"/>
     </row>
     <row r="114" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -3244,6 +3248,62 @@
       <c r="C117" s="24"/>
       <c r="D117" s="24"/>
       <c r="E117" s="24"/>
+    </row>
+    <row r="118" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A118" s="24"/>
+      <c r="B118" s="24"/>
+      <c r="C118" s="24"/>
+      <c r="D118" s="24"/>
+      <c r="E118" s="24"/>
+    </row>
+    <row r="119" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A119" s="24"/>
+      <c r="B119" s="24"/>
+      <c r="C119" s="24"/>
+      <c r="D119" s="24"/>
+      <c r="E119" s="24"/>
+    </row>
+    <row r="120" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A120" s="24"/>
+      <c r="B120" s="24"/>
+      <c r="C120" s="24"/>
+      <c r="D120" s="24"/>
+      <c r="E120" s="24"/>
+    </row>
+    <row r="121" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A121" s="24"/>
+      <c r="B121" s="24"/>
+      <c r="C121" s="24"/>
+      <c r="D121" s="24"/>
+      <c r="E121" s="24"/>
+    </row>
+    <row r="122" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A122" s="24"/>
+      <c r="B122" s="24"/>
+      <c r="C122" s="24"/>
+      <c r="D122" s="24"/>
+      <c r="E122" s="24"/>
+    </row>
+    <row r="123" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A123" s="24"/>
+      <c r="B123" s="24"/>
+      <c r="C123" s="24"/>
+      <c r="D123" s="24"/>
+      <c r="E123" s="24"/>
+    </row>
+    <row r="124" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A124" s="24"/>
+      <c r="B124" s="24"/>
+      <c r="C124" s="24"/>
+      <c r="D124" s="24"/>
+      <c r="E124" s="24"/>
+    </row>
+    <row r="125" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A125" s="24"/>
+      <c r="B125" s="24"/>
+      <c r="C125" s="24"/>
+      <c r="D125" s="24"/>
+      <c r="E125" s="24"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>